<commit_message>
fix: language detection + professional English flow
</commit_message>
<xml_diff>
--- a/scraper/downloads/yad2_page_1.xlsx
+++ b/scraper/downloads/yad2_page_1.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c t="inlineStr" r="E8">
         <is>
-          <t xml:space="preserve">/52</t>
+          <t xml:space="preserve">/53</t>
         </is>
       </c>
       <c t="inlineStr" r="F8">
@@ -693,12 +693,12 @@
       </c>
       <c t="inlineStr" r="H8">
         <is>
-          <t xml:space="preserve">190מ״ר</t>
+          <t xml:space="preserve">164מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="I8">
         <is>
-          <t xml:space="preserve">מרפסת: 24מ״ר</t>
+          <t xml:space="preserve">מרפסת: 12מ״רמרפסת: 15מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J8">
@@ -718,11 +718,11 @@
       </c>
       <c t="inlineStr" r="N8">
         <is>
-          <t xml:space="preserve">מתן (052) 537-1059</t>
+          <t xml:space="preserve">מתן(052) 537-1059</t>
         </is>
       </c>
       <c r="O8" s="63">
-        <v>16500000</v>
+        <v>15500000</v>
       </c>
       <c t="inlineStr" r="R8">
         <is>
@@ -754,7 +754,7 @@
       </c>
       <c t="inlineStr" r="E9">
         <is>
-          <t xml:space="preserve">/53</t>
+          <t xml:space="preserve">/52</t>
         </is>
       </c>
       <c t="inlineStr" r="F9">
@@ -767,12 +767,12 @@
       </c>
       <c t="inlineStr" r="H9">
         <is>
-          <t xml:space="preserve">164מ״ר</t>
+          <t xml:space="preserve">190מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="I9">
         <is>
-          <t xml:space="preserve">מרפסת: 12מ״רמרפסת: 15מ״ר</t>
+          <t xml:space="preserve">מרפסת: 24מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J9">
@@ -792,11 +792,11 @@
       </c>
       <c t="inlineStr" r="N9">
         <is>
-          <t xml:space="preserve">מתן(052) 537-1059</t>
+          <t xml:space="preserve">מתן (052) 537-1059</t>
         </is>
       </c>
       <c r="O9" s="63">
-        <v>15500000</v>
+        <v>16500000</v>
       </c>
       <c t="inlineStr" r="R9">
         <is>
@@ -1408,26 +1408,33 @@
       </c>
       <c t="inlineStr" r="C18">
         <is>
-          <t xml:space="preserve">אושה</t>
+          <t xml:space="preserve">אוסישקין</t>
         </is>
       </c>
       <c r="D18" s="65">
-        <v>7</v>
-      </c>
-      <c r="E18" s="65">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c t="inlineStr" r="E18">
+        <is>
+          <t xml:space="preserve">/40</t>
+        </is>
       </c>
       <c t="inlineStr" r="F18">
         <is>
-          <t xml:space="preserve">בית פרטי</t>
-        </is>
-      </c>
-      <c r="G18" s="65">
-        <v>0</v>
+          <t xml:space="preserve">דירת גן</t>
+        </is>
+      </c>
+      <c t="n" r="G18">
+        <v>3.5</v>
       </c>
       <c t="inlineStr" r="H18">
         <is>
-          <t xml:space="preserve">300מ״ר</t>
+          <t xml:space="preserve">71מ״ר</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I18">
+        <is>
+          <t xml:space="preserve">מרפסת: 12מ״רגינה: 50מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J18">
@@ -1437,16 +1444,26 @@
       </c>
       <c t="inlineStr" r="K18">
         <is>
-          <t xml:space="preserve">ללא מחסן</t>
+          <t xml:space="preserve">יש מחסן</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="L18">
+        <is>
+          <t xml:space="preserve">דרום מזרח מערב</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="M18">
+        <is>
+          <t xml:space="preserve">חזית עורף</t>
         </is>
       </c>
       <c t="inlineStr" r="N18">
         <is>
-          <t xml:space="preserve">אהרון וולק (054) 497-8899</t>
+          <t xml:space="preserve">מתי כוחיי(050) 620-7066דבורה(050) 621-8349</t>
         </is>
       </c>
       <c r="O18" s="63">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c t="inlineStr" r="R18">
         <is>
@@ -1455,7 +1472,7 @@
       </c>
       <c t="inlineStr" r="S18">
         <is>
-          <t xml:space="preserve">מנחם אוריאל13-11-2024</t>
+          <t xml:space="preserve">אריה טאו15-06-2026</t>
         </is>
       </c>
     </row>
@@ -1470,26 +1487,26 @@
       </c>
       <c t="inlineStr" r="C19">
         <is>
-          <t xml:space="preserve">אחד העם</t>
+          <t xml:space="preserve">אושה</t>
         </is>
       </c>
       <c r="D19" s="65">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="E19" s="65">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F19">
         <is>
-          <t xml:space="preserve">דירה</t>
+          <t xml:space="preserve">בית פרטי</t>
         </is>
       </c>
       <c r="G19" s="65">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="H19">
         <is>
-          <t xml:space="preserve">70מ״ר</t>
+          <t xml:space="preserve">300מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J19">
@@ -1504,11 +1521,11 @@
       </c>
       <c t="inlineStr" r="N19">
         <is>
-          <t xml:space="preserve">סינגר סיימון</t>
-        </is>
-      </c>
-      <c r="O19" s="65">
-        <v>0</v>
+          <t xml:space="preserve">אהרון וולק (054) 497-8899</t>
+        </is>
+      </c>
+      <c r="O19" s="63">
+        <v>50000</v>
       </c>
       <c t="inlineStr" r="R19">
         <is>
@@ -1517,7 +1534,7 @@
       </c>
       <c t="inlineStr" r="S19">
         <is>
-          <t xml:space="preserve">רבקה בן זקן04-11-2024</t>
+          <t xml:space="preserve">מנחם אוריאל13-11-2024</t>
         </is>
       </c>
     </row>
@@ -1532,11 +1549,11 @@
       </c>
       <c t="inlineStr" r="C20">
         <is>
-          <t xml:space="preserve">איתמר בן אבי</t>
+          <t xml:space="preserve">אחד העם</t>
         </is>
       </c>
       <c r="D20" s="65">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="E20" s="65">
         <v>0</v>
@@ -1547,18 +1564,13 @@
         </is>
       </c>
       <c r="G20" s="65">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="H20">
         <is>
           <t xml:space="preserve">70מ״ר</t>
         </is>
       </c>
-      <c t="inlineStr" r="I20">
-        <is>
-          <t xml:space="preserve">מרפסת: 5מ״ר</t>
-        </is>
-      </c>
       <c t="inlineStr" r="J20">
         <is>
           <t xml:space="preserve">ללא חניה</t>
@@ -1571,11 +1583,11 @@
       </c>
       <c t="inlineStr" r="N20">
         <is>
-          <t xml:space="preserve">יהושוע רוז(053) 478-5082</t>
-        </is>
-      </c>
-      <c r="O20" s="63">
-        <v>4150000</v>
+          <t xml:space="preserve">סינגר סיימון</t>
+        </is>
+      </c>
+      <c r="O20" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="R20">
         <is>
@@ -1584,7 +1596,7 @@
       </c>
       <c t="inlineStr" r="S20">
         <is>
-          <t xml:space="preserve">רבקה בן זקן29-10-2025</t>
+          <t xml:space="preserve">רבקה בן זקן04-11-2024</t>
         </is>
       </c>
     </row>
@@ -1599,16 +1611,14 @@
       </c>
       <c t="inlineStr" r="C21">
         <is>
-          <t xml:space="preserve">אלכסנדריון</t>
+          <t xml:space="preserve">איתמר בן אבי</t>
         </is>
       </c>
       <c r="D21" s="65">
-        <v>15</v>
-      </c>
-      <c t="inlineStr" r="E21">
-        <is>
-          <t xml:space="preserve">/31</t>
-        </is>
+        <v>6</v>
+      </c>
+      <c r="E21" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F21">
         <is>
@@ -1616,11 +1626,16 @@
         </is>
       </c>
       <c r="G21" s="65">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="H21">
         <is>
-          <t xml:space="preserve">155מ״ר</t>
+          <t xml:space="preserve">70מ״ר</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I21">
+        <is>
+          <t xml:space="preserve">מרפסת: 5מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J21">
@@ -1635,11 +1650,11 @@
       </c>
       <c t="inlineStr" r="N21">
         <is>
-          <t xml:space="preserve">אושי - מתווך(050) 286-9312</t>
+          <t xml:space="preserve">יהושוע רוז(053) 478-5082</t>
         </is>
       </c>
       <c r="O21" s="63">
-        <v>4700000</v>
+        <v>4150000</v>
       </c>
       <c t="inlineStr" r="R21">
         <is>
@@ -1648,7 +1663,7 @@
       </c>
       <c t="inlineStr" r="S21">
         <is>
-          <t xml:space="preserve">מנחם אוריאל16-02-2026</t>
+          <t xml:space="preserve">רבקה בן זקן29-10-2025</t>
         </is>
       </c>
     </row>
@@ -1663,31 +1678,28 @@
       </c>
       <c t="inlineStr" r="C22">
         <is>
-          <t xml:space="preserve">אלפסי</t>
+          <t xml:space="preserve">אלכסנדריון</t>
         </is>
       </c>
       <c r="D22" s="65">
-        <v>29</v>
-      </c>
-      <c r="E22" s="65">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c t="inlineStr" r="E22">
+        <is>
+          <t xml:space="preserve">/31</t>
+        </is>
       </c>
       <c t="inlineStr" r="F22">
         <is>
           <t xml:space="preserve">דירה</t>
         </is>
       </c>
-      <c t="n" r="G22">
-        <v>4.5</v>
+      <c r="G22" s="65">
+        <v>6</v>
       </c>
       <c t="inlineStr" r="H22">
         <is>
-          <t xml:space="preserve">121מ״ר</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I22">
-        <is>
-          <t xml:space="preserve">מרפסת: 14מ״ר</t>
+          <t xml:space="preserve">155מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J22">
@@ -1702,11 +1714,11 @@
       </c>
       <c t="inlineStr" r="N22">
         <is>
-          <t xml:space="preserve">moshe@orencohengroup.com</t>
-        </is>
-      </c>
-      <c r="O22" s="65">
-        <v>0</v>
+          <t xml:space="preserve">אושי - מתווך(050) 286-9312</t>
+        </is>
+      </c>
+      <c r="O22" s="63">
+        <v>4700000</v>
       </c>
       <c t="inlineStr" r="R22">
         <is>
@@ -1715,7 +1727,7 @@
       </c>
       <c t="inlineStr" r="S22">
         <is>
-          <t xml:space="preserve">אורן כהן04-11-2024</t>
+          <t xml:space="preserve">מנחם אוריאל16-02-2026</t>
         </is>
       </c>
     </row>
@@ -1736,8 +1748,10 @@
       <c r="D23" s="65">
         <v>29</v>
       </c>
-      <c r="E23" s="65">
-        <v>0</v>
+      <c t="inlineStr" r="E23">
+        <is>
+          <t xml:space="preserve">/51</t>
+        </is>
       </c>
       <c t="inlineStr" r="F23">
         <is>
@@ -1745,35 +1759,35 @@
         </is>
       </c>
       <c r="G23" s="65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c t="inlineStr" r="H23">
         <is>
-          <t xml:space="preserve">115.5מ״ר</t>
+          <t xml:space="preserve">121מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="I23">
         <is>
-          <t xml:space="preserve">מרפסת: 18.3מ״ר</t>
+          <t xml:space="preserve">מרפסת: 18.8מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J23">
         <is>
-          <t xml:space="preserve">ללא חניה</t>
+          <t xml:space="preserve">1חניות</t>
         </is>
       </c>
       <c t="inlineStr" r="K23">
         <is>
-          <t xml:space="preserve">ללא מחסן</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="N23">
-        <is>
-          <t xml:space="preserve">moshe@orencohengroup.com</t>
-        </is>
-      </c>
-      <c r="O23" s="65">
-        <v>0</v>
+          <t xml:space="preserve">יש מחסן</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="L23">
+        <is>
+          <t xml:space="preserve">דרום מזרח מערב</t>
+        </is>
+      </c>
+      <c r="O23" s="63">
+        <v>10300000</v>
       </c>
       <c t="inlineStr" r="R23">
         <is>
@@ -1782,7 +1796,7 @@
       </c>
       <c t="inlineStr" r="S23">
         <is>
-          <t xml:space="preserve">אורן כהן04-11-2024</t>
+          <t xml:space="preserve">משה קולטון29-06-2025</t>
         </is>
       </c>
     </row>
@@ -1803,10 +1817,8 @@
       <c r="D24" s="65">
         <v>29</v>
       </c>
-      <c t="inlineStr" r="E24">
-        <is>
-          <t xml:space="preserve">/51</t>
-        </is>
+      <c r="E24" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F24">
         <is>
@@ -1814,35 +1826,35 @@
         </is>
       </c>
       <c r="G24" s="65">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c t="inlineStr" r="H24">
         <is>
-          <t xml:space="preserve">121מ״ר</t>
+          <t xml:space="preserve">115.5מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="I24">
         <is>
-          <t xml:space="preserve">מרפסת: 18.8מ״ר</t>
+          <t xml:space="preserve">מרפסת: 18.3מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J24">
         <is>
-          <t xml:space="preserve">1חניות</t>
+          <t xml:space="preserve">ללא חניה</t>
         </is>
       </c>
       <c t="inlineStr" r="K24">
         <is>
-          <t xml:space="preserve">יש מחסן</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="L24">
-        <is>
-          <t xml:space="preserve">דרום מזרח מערב</t>
-        </is>
-      </c>
-      <c r="O24" s="63">
-        <v>10300000</v>
+          <t xml:space="preserve">ללא מחסן</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="N24">
+        <is>
+          <t xml:space="preserve">moshe@orencohengroup.com</t>
+        </is>
+      </c>
+      <c r="O24" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="R24">
         <is>
@@ -1851,7 +1863,7 @@
       </c>
       <c t="inlineStr" r="S24">
         <is>
-          <t xml:space="preserve">משה קולטון29-06-2025</t>
+          <t xml:space="preserve">אורן כהן04-11-2024</t>
         </is>
       </c>
     </row>
@@ -1990,16 +2002,14 @@
       </c>
       <c t="inlineStr" r="C27">
         <is>
-          <t xml:space="preserve">ארלוזורוב</t>
+          <t xml:space="preserve">אלפסי</t>
         </is>
       </c>
       <c r="D27" s="65">
-        <v>13</v>
-      </c>
-      <c t="inlineStr" r="E27">
-        <is>
-          <t xml:space="preserve">/53</t>
-        </is>
+        <v>29</v>
+      </c>
+      <c r="E27" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F27">
         <is>
@@ -2007,16 +2017,16 @@
         </is>
       </c>
       <c t="n" r="G27">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c t="inlineStr" r="H27">
         <is>
-          <t xml:space="preserve">59מ״ר</t>
+          <t xml:space="preserve">121מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="I27">
         <is>
-          <t xml:space="preserve">מרפסת: 12מ״ר</t>
+          <t xml:space="preserve">מרפסת: 14מ״ר</t>
         </is>
       </c>
       <c t="inlineStr" r="J27">
@@ -2026,21 +2036,16 @@
       </c>
       <c t="inlineStr" r="K27">
         <is>
-          <t xml:space="preserve">יש מחסן</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="L27">
-        <is>
-          <t xml:space="preserve">צפון מזרח מערב</t>
+          <t xml:space="preserve">ללא מחסן</t>
         </is>
       </c>
       <c t="inlineStr" r="N27">
         <is>
-          <t xml:space="preserve">ארז נתנאלי- לא לפנות(054) 743-3889שוכרת- ניצן(054) 492-2952</t>
-        </is>
-      </c>
-      <c r="O27" s="63">
-        <v>5490000</v>
+          <t xml:space="preserve">moshe@orencohengroup.com</t>
+        </is>
+      </c>
+      <c r="O27" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="R27">
         <is>
@@ -2049,7 +2054,7 @@
       </c>
       <c t="inlineStr" r="S27">
         <is>
-          <t xml:space="preserve">אורן כהן06-01-2025</t>
+          <t xml:space="preserve">אורן כהן04-11-2024</t>
         </is>
       </c>
     </row>

</xml_diff>